<commit_message>
Check pipeline continiuty in pipe network
</commit_message>
<xml_diff>
--- a/Documentation/Friction loss.xlsx
+++ b/Documentation/Friction loss.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\admin\Lytrose\repos\Pump-Master-Pro\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{30CAC74D-6EB5-4C0B-ACC8-CF643B930DAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{94CAD49E-5D71-48EF-AB7F-8DD886DB6A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="3" activeTab="4" xr2:uid="{288D667A-AE77-4017-BD75-930C7D5D6DD0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="6" xr2:uid="{288D667A-AE77-4017-BD75-930C7D5D6DD0}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Sanitize friction calcs on pipe network
</commit_message>
<xml_diff>
--- a/Documentation/Friction loss.xlsx
+++ b/Documentation/Friction loss.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\admin\Lytrose\repos\Pump-Master-Pro\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{94CAD49E-5D71-48EF-AB7F-8DD886DB6A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785CD414-1CD3-464D-B912-0400FA997A5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="6" xr2:uid="{288D667A-AE77-4017-BD75-930C7D5D6DD0}"/>
+    <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12336" firstSheet="1" activeTab="5" xr2:uid="{288D667A-AE77-4017-BD75-930C7D5D6DD0}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -1759,7 +1759,7 @@
         <v>38</v>
       </c>
       <c r="B15" s="3">
-        <v>1</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="B16" s="4">
         <f>B15*0.000001</f>
-        <v>9.9999999999999995E-7</v>
+        <v>1.2299999999999999E-6</v>
       </c>
     </row>
   </sheetData>
@@ -1803,7 +1803,7 @@
         <v>43</v>
       </c>
       <c r="B4" s="3">
-        <v>36</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1811,7 +1811,7 @@
         <v>44</v>
       </c>
       <c r="B5" s="3">
-        <v>100</v>
+        <v>85.56</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1819,7 +1819,7 @@
         <v>45</v>
       </c>
       <c r="B6" s="3">
-        <v>100</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1827,7 +1827,7 @@
         <v>46</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>47</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="B8" s="4">
         <f>IFERROR(VLOOKUP(B7,Reference!$A$2:$B$10,2,FALSE),0.046)</f>
-        <v>4.5999999999999999E-2</v>
+        <v>7.0000000000000001E-3</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1851,9 +1851,9 @@
       <c r="A10" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="4" t="e">
+      <c r="B10" s="4">
         <f>Minor_Losses!$B$18</f>
-        <v>#VALUE!</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1861,7 +1861,7 @@
         <v>51</v>
       </c>
       <c r="B11" s="3">
-        <v>1</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1898,7 +1898,7 @@
         <v>56</v>
       </c>
       <c r="B17" s="3">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -1906,7 +1906,7 @@
         <v>57</v>
       </c>
       <c r="B18" s="3">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="B22" s="4">
         <f>IF(B3="Slurry",(B16+(B17/100/B15)/((B17/100/B15)+((1-B17/100)/B16))*(B15-B16))*Fluid_Props!$B$5*B11,B11*Fluid_Props!$B$5)</f>
-        <v>999.48800000000006</v>
+        <v>1229.37024</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="B23" s="4">
         <f>B4/3600</f>
-        <v>0.01</v>
+        <v>2.7777777777777776E-2</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B24" s="4">
         <f>B5/1000</f>
-        <v>0.1</v>
+        <v>8.5559999999999997E-2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B25" s="4">
         <f>PI()*B24^2/4</f>
-        <v>7.8539816339744835E-3</v>
+        <v>5.7495179365660417E-3</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B26" s="4">
         <f>B23/B25</f>
-        <v>1.2732395447351625</v>
+        <v>4.8313229185903435</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -1974,25 +1974,25 @@
       </c>
       <c r="B27" s="4">
         <f>B26^2/(2*9.80665)</f>
-        <v>8.2655082942564698E-2</v>
+        <v>1.1900945350194161</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="4" t="e">
-        <f>B27*B24/B20</f>
-        <v>#DIV/0!</v>
+      <c r="B28" s="4">
+        <f>B27*B24/B21</f>
+        <v>100142.56606295692</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="4" t="e">
+      <c r="B29" s="4" t="str">
         <f>IF(B28&lt;2300,"Laminar",IF(B28&lt;4000,"Transitional","Turbulent"))</f>
-        <v>#DIV/0!</v>
+        <v>Turbulent</v>
       </c>
     </row>
   </sheetData>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="B3" s="4">
         <f>Pipe_Inputs!$B$24</f>
-        <v>0.1</v>
+        <v>8.5559999999999997E-2</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="B4" s="4">
         <f>Pipe_Inputs!$B$6</f>
-        <v>100</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2038,16 +2038,16 @@
       </c>
       <c r="B5" s="4">
         <f>Pipe_Inputs!$B$8</f>
-        <v>4.5999999999999999E-2</v>
+        <v>7.0000000000000001E-3</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="4" t="e">
+      <c r="B6" s="4">
         <f>Pipe_Inputs!$B$10</f>
-        <v>#VALUE!</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="B7" s="4">
         <f>Pipe_Inputs!$B$23</f>
-        <v>0.01</v>
+        <v>2.7777777777777776E-2</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="B8" s="4">
         <f>Pipe_Inputs!$B$26</f>
-        <v>1.2732395447351625</v>
+        <v>4.8313229185903435</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2081,18 +2081,18 @@
       <c r="A10" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="4" t="e">
+      <c r="B10" s="4">
         <f>Pipe_Inputs!$B$28</f>
-        <v>#DIV/0!</v>
+        <v>100142.56606295692</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="4" t="e">
+      <c r="B11" s="4" t="str">
         <f>Pipe_Inputs!$B$29</f>
-        <v>#DIV/0!</v>
+        <v>Turbulent</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -2113,27 +2113,27 @@
       <c r="A15" t="s">
         <v>74</v>
       </c>
-      <c r="B15" s="4" t="e">
+      <c r="B15" s="4">
         <f>IF(B10&gt;0,64/B10,0.02)</f>
-        <v>#DIV/0!</v>
+        <v>6.3908887615047661E-4</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>75</v>
       </c>
-      <c r="B16" s="4" t="e">
+      <c r="B16" s="4">
         <f>B15*(1-(B10-2300)/1700)+B14*((B10-2300)/1700)</f>
-        <v>#DIV/0!</v>
+        <v>0.34398440884124504</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="4" t="e">
+      <c r="B17" s="4">
         <f>IF(B10&lt;2300,B15,IF(B10&lt;4000,B16,B14))</f>
-        <v>#DIV/0!</v>
+        <v>6.6046626282236448E-3</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -2145,9 +2145,9 @@
       <c r="A20" t="s">
         <v>78</v>
       </c>
-      <c r="B20" s="4" t="e">
-        <f>B18*(B3/B2)*(B7^2)/(2*9.80665)</f>
-        <v>#DIV/0!</v>
+      <c r="B20" s="4">
+        <f>B17*(B4/B3)*(B7^2)/(2*9.80665)</f>
+        <v>9.7179389862129327E-5</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -2159,9 +2159,9 @@
       <c r="A23" t="s">
         <v>80</v>
       </c>
-      <c r="B23" s="4" t="e">
+      <c r="B23" s="4">
         <f>B6*(B8^2)/(2*9.80665)</f>
-        <v>#VALUE!</v>
+        <v>0.23801890700388326</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -2173,9 +2173,9 @@
       <c r="A26" t="s">
         <v>82</v>
       </c>
-      <c r="B26" s="4" t="e">
+      <c r="B26" s="4">
         <f>B20+B23</f>
-        <v>#DIV/0!</v>
+        <v>0.23811608639374537</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -2191,9 +2191,9 @@
       <c r="A28" t="s">
         <v>84</v>
       </c>
-      <c r="B28" s="4" t="e">
+      <c r="B28" s="4">
         <f>B26+B27</f>
-        <v>#DIV/0!</v>
+        <v>0.23811608639374537</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -2205,9 +2205,9 @@
       <c r="A31" t="s">
         <v>86</v>
       </c>
-      <c r="B31" s="4" t="e">
+      <c r="B31" s="4">
         <f>8/(9.80665*PI()^2*B3^4)*(B17*B4/B3+B9)</f>
-        <v>#DIV/0!</v>
+        <v>3809.9254870127816</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -2222,9 +2222,9 @@
       <c r="A33" t="s">
         <v>88</v>
       </c>
-      <c r="B33" s="4" t="e">
+      <c r="B33" s="4">
         <f>B31*B9^2</f>
-        <v>#DIV/0!</v>
+        <v>3.9389777204392666E-9</v>
       </c>
     </row>
   </sheetData>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B3" s="4">
         <f>Pipe_Inputs!$B$24</f>
-        <v>0.1</v>
+        <v>8.5559999999999997E-2</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B4" s="4">
         <f>Pipe_Inputs!$B$6</f>
-        <v>100</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="B5" s="4">
         <f>Pipe_Inputs!$B$23</f>
-        <v>0.01</v>
+        <v>2.7777777777777776E-2</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="B6" s="4" t="str">
         <f>Pipe_Inputs!$B$7</f>
-        <v>commercial_steel</v>
+        <v>hdpe</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B7" s="4">
         <f>IFERROR(VLOOKUP(B6,Reference!$E$2:$F$10,2,FALSE),120)</f>
-        <v>120</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2300,9 +2300,9 @@
       <c r="A10" t="s">
         <v>78</v>
       </c>
-      <c r="B10" s="4" t="e">
-        <f>10.67*B4*B6^(-1.852)*B3^(-4.87)*B5^1.852</f>
-        <v>#VALUE!</v>
+      <c r="B10" s="4">
+        <f>10.67*B4*B7^(-1.852)*B3^(-4.87)*B5^1.852</f>
+        <v>7.5206324734727481</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -2314,9 +2314,9 @@
       <c r="A13" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="4" t="e">
+      <c r="B13" s="4">
         <f>Pipe_Inputs!$B$10</f>
-        <v>#VALUE!</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -2331,27 +2331,27 @@
       <c r="A15" t="s">
         <v>93</v>
       </c>
-      <c r="B15" s="4" t="e">
+      <c r="B15" s="4">
         <f>B13*(B3/B14)</f>
-        <v>#VALUE!</v>
+        <v>0.85559999999999992</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>94</v>
       </c>
-      <c r="B16" s="4" t="e">
+      <c r="B16" s="4">
         <f>B4+B15</f>
-        <v>#VALUE!</v>
+        <v>32.855600000000003</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>95</v>
       </c>
-      <c r="B17" s="4" t="e">
-        <f>10.67*B15*B8^(-1.852)*B5^(-4.87)*B7^1.852</f>
-        <v>#VALUE!</v>
+      <c r="B17" s="4">
+        <f>10.67*B15*B7^(-1.852)*B3^(-4.87)*B5^1.852</f>
+        <v>0.2010829107594776</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -2363,18 +2363,18 @@
       <c r="A20" t="s">
         <v>82</v>
       </c>
-      <c r="B20" s="4" t="e">
+      <c r="B20" s="4">
         <f>B10+B16</f>
-        <v>#VALUE!</v>
+        <v>40.376232473472754</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="4" t="e">
+      <c r="B21" s="4">
         <f>B20+Pipe_Inputs!$B$9</f>
-        <v>#VALUE!</v>
+        <v>40.376232473472754</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -2386,9 +2386,9 @@
       <c r="A24" t="s">
         <v>96</v>
       </c>
-      <c r="B24" s="4" t="e">
-        <f>10.67*B16*B5^(-1.852)*B2^(-4.87)</f>
-        <v>#VALUE!</v>
+      <c r="B24" s="4">
+        <f>10.67*B16*B5^(-1.852)*B21^(-4.87)</f>
+        <v>4.0291500852538365E-3</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -2403,9 +2403,9 @@
       <c r="A26" t="s">
         <v>97</v>
       </c>
-      <c r="B26" s="4" t="e">
-        <f>B24*B2^B25</f>
-        <v>#VALUE!</v>
+      <c r="B26" s="4">
+        <f>B24*B21^B25</f>
+        <v>3.7997796486350546</v>
       </c>
     </row>
   </sheetData>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="B6" s="4">
         <f>Pipe_Inputs!$B$17</f>
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="B7" s="4">
         <f>Pipe_Inputs!$B$18</f>
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B8" s="4">
         <f>Pipe_Inputs!$B$24</f>
-        <v>0.1</v>
+        <v>8.5559999999999997E-2</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B9" s="4">
         <f>Pipe_Inputs!$B$26</f>
-        <v>1.2732395447351625</v>
+        <v>4.8313229185903435</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -2499,9 +2499,9 @@
       <c r="A11" t="s">
         <v>78</v>
       </c>
-      <c r="B11" s="4" t="e">
+      <c r="B11" s="4">
         <f>Darcy_Weisbach!$B$20</f>
-        <v>#DIV/0!</v>
+        <v>9.7179389862129327E-5</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="B12" s="4">
         <f>Pipe_Inputs!$B$6</f>
-        <v>100</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="B28" s="4">
         <f>B27*SQRT(2*9.80665*B6*(B6-B7)/B7)</f>
-        <v>413.26717281570205</v>
+        <v>383.68731905354917</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="B29" s="4">
         <f>B6/B28</f>
-        <v>6.0493553914936375E-2</v>
+        <v>7.8188666943702301E-2</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="B34" s="4">
         <f>(4/3)*9.80665*B16*(B9-B10)/B17^2</f>
-        <v>9.0708632931632699E-3</v>
+        <v>3.4419521193218082E-2</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="B35" s="4">
         <f>B4^2*SQRT(B34)/(9.80665*B5*(B4-B5))</f>
-        <v>4.1334381065575423E-2</v>
+        <v>8.0517362514768556E-2</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="B36" s="4">
         <f>82*B35^(-1.5)</f>
-        <v>9757.6827520574971</v>
+        <v>3589.0502740507536</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -2699,18 +2699,18 @@
       <c r="A39" t="s">
         <v>80</v>
       </c>
-      <c r="B39" s="4" t="e">
+      <c r="B39" s="4">
         <f>Darcy_Weisbach!$B$23</f>
-        <v>#VALUE!</v>
+        <v>0.23801890700388326</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
         <v>82</v>
       </c>
-      <c r="B40" s="4" t="e">
+      <c r="B40" s="4">
         <f>B38+B39</f>
-        <v>#VALUE!</v>
+        <v>0.23801890700388326</v>
       </c>
     </row>
   </sheetData>
@@ -2755,11 +2755,11 @@
         <v>0.9</v>
       </c>
       <c r="C4" s="3">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4" t="e">
-        <f t="shared" ref="D4:D14" si="0">B3*C3</f>
-        <v>#VALUE!</v>
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <f>B4*C4</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2773,8 +2773,8 @@
         <v>0</v>
       </c>
       <c r="D5" s="4">
-        <f t="shared" si="0"/>
-        <v>1.8</v>
+        <f t="shared" ref="D5:D14" si="0">B5*C5</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="D8" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="D9" s="4">
         <f t="shared" si="0"/>
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2928,9 +2928,9 @@
       <c r="A18" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B18" s="4" t="e">
+      <c r="B18" s="4">
         <f>SUM(D4:D14)+D16</f>
-        <v>#VALUE!</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="19" spans="1:2">

</xml_diff>